<commit_message>
docs(audit): mise à jour de la matrice de risques — 16/16 actionnables traités
Régénération de la matrice Excel après déploiement des patches P1+P2+P3 :
- CRIT-1, HIGH-1, HIGH-3, HIGH-4 (P1) → Traité
- HIGH-2, MED-3, MED-4, MED-5 (P2) → Traité
- MED-1, MED-2, MED-6, MED-7, LOW-1 à LOW-6 (P3) → Traité
- INFO-1 à INFO-4 → Informatif (aucune action requise)

Tests de non-régression : 107 tests (P1+P2+P3) passent.
Migrations déployables : 20260708000000, 20260708010000, 20260708020000.

Référence audit : AUDIT-2026-007
</commit_message>
<xml_diff>
--- a/docs/audit/matrice-risques-2026-07-07.xlsx
+++ b/docs/audit/matrice-risques-2026-07-07.xlsx
@@ -67,7 +67,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00C0392B"/>
+      <color rgb="001B7D46"/>
       <sz val="10"/>
     </font>
     <font>
@@ -85,13 +85,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00D4820A"/>
+      <color rgb="00C0392B"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001B7D46"/>
+      <color rgb="00D4820A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -120,7 +120,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDEDEC"/>
+        <fgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
     <fill>
@@ -155,12 +155,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF9E7"/>
+        <fgColor rgb="00FDEDEC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F5E9"/>
+        <fgColor rgb="00FEF9E7"/>
       </patternFill>
     </fill>
     <fill>
@@ -267,16 +267,16 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -676,7 +676,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Audit du 7 juillet 2026 · 22 findings (1 critique, 4 élevés, 7 moyens, 6 faibles, 4 infos) · Référence AUDIT-2026-007</t>
+          <t>Audit du 7 juillet 2026 · 22 findings · 16/16 actionnables traités (P1+P2+P3) · 4 informatifs · Référence AUDIT-2026-007</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M6" s="7" t="inlineStr"/>
@@ -865,7 +865,7 @@
       </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M7" s="12" t="inlineStr"/>
@@ -925,7 +925,7 @@
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M8" s="7" t="inlineStr"/>
@@ -985,7 +985,7 @@
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M9" s="12" t="inlineStr"/>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr"/>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M11" s="12" t="inlineStr"/>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr"/>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M13" s="12" t="inlineStr"/>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M14" s="7" t="inlineStr"/>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M15" s="12" t="inlineStr"/>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M16" s="7" t="inlineStr"/>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M17" s="12" t="inlineStr"/>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>Supprimer la ligne GRANT morte.</t>
+          <t>Supprimer la ligne GRANT morte. No-op en DB (le GRANT a échoué silencieusement).</t>
         </is>
       </c>
       <c r="I18" s="7" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M18" s="7" t="inlineStr"/>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M19" s="12" t="inlineStr"/>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M20" s="7" t="inlineStr"/>
@@ -1705,7 +1705,7 @@
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M21" s="12" t="inlineStr"/>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M22" s="7" t="inlineStr"/>
@@ -1825,7 +1825,7 @@
       </c>
       <c r="L23" s="8" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Traité</t>
         </is>
       </c>
       <c r="M23" s="12" t="inlineStr"/>

</xml_diff>